<commit_message>
Improve math model v1.4.0: correct two-phase fault, add fault types and IEC factors
- fix two-phase fault current: add sqrt(3) factor (Ik2 ≈ 0.866·Ik3)
- add double-line-to-ground fault (Ik1.1) and earth current
- voltage factor c per GOST R 52735 / IEC 60909 (column c, default 1.1)
- transition/arc resistance Rf in fault loop (column Rf)
- parallel branches via column Parallel (parallel within group, then series)
- breaking current (with asymmetry) and thermal equivalent current
- new modules: func_fault_currents, func_breaking_thermal, func_pu_to_ka, sc_series_parallel
- wire into main_calc_sc, oct_sc_menu, run_points; extend reports (txt/Word/CSV)
- update verify_sc_suite (18 tests), INSTRUKCIYA.md, version to 1.4.0
</commit_message>
<xml_diff>
--- a/network_parameters.xlsx
+++ b/network_parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projekt\Maga\SC_Calculator_MATLAB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBB109C0-FC59-4522-82C6-1587FA1C4130}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A725EDB-8F9A-4409-80D1-8AA4724542E1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4716" yWindow="2448" windowWidth="17280" windowHeight="8880" xr2:uid="{9A2AD5B8-86FE-4B19-8A10-42F89054F8D7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9A2AD5B8-86FE-4B19-8A10-42F89054F8D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -67,16 +67,35 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -84,12 +103,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -406,48 +442,52 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7D8722A-36EB-4996-8498-9D240087A3A1}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" ht="44.4" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="2" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
         <v>0.5</v>
       </c>
-      <c r="C2">
-        <v>8.5</v>
-      </c>
-      <c r="D2">
-        <v>0.8</v>
-      </c>
-      <c r="E2">
-        <v>6.5</v>
-      </c>
-      <c r="F2">
-        <v>10</v>
+      <c r="C2" s="2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="E2" s="2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F2" s="2">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>